<commit_message>
Adding latest update of the model
</commit_message>
<xml_diff>
--- a/Sets-TIMES-AFOLU.xlsx
+++ b/Sets-TIMES-AFOLU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://politoit-my.sharepoint.com/personal/daniele_mosso_polito_it/Documents/Desktop/EML/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git-repositories\TIMES-AFOLU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{5E61A486-1F70-4BAD-B132-FEA29753E527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53A9F48D-1765-4804-AE33-DCE94E38A439}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7CAA76-5115-4E96-91BA-CB06CF720CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proc_Sets_AFO" sheetId="11" r:id="rId1"/>
@@ -83,9 +83,6 @@
     <t>Forest</t>
   </si>
   <si>
-    <t>AFOFRSNRGF_E1,AFOFRSPGF_E1</t>
-  </si>
-  <si>
     <t>All Livestock</t>
   </si>
   <si>
@@ -168,6 +165,9 @@
   </si>
   <si>
     <t>Process Sets Definition for AFOLU</t>
+  </si>
+  <si>
+    <t>AFOFRSNRGFE0</t>
   </si>
 </sst>
 </file>
@@ -372,7 +372,7 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -386,6 +386,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="32">
     <cellStyle name="a_Calc_Outputs" xfId="12" xr:uid="{F3B733CB-9C19-4D45-9722-13862E8D6D18}"/>
@@ -698,24 +699,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEFF0143-B648-4A8C-A514-3939749F766D}">
   <dimension ref="B1:E16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="70.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="70.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="93" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" s="4" customFormat="1" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:5" s="4" customFormat="1" ht="23.5" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -723,7 +724,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="2:5" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
@@ -737,7 +738,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -748,7 +749,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>8</v>
       </c>
@@ -759,114 +760,114 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" t="s">
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" t="s">
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
         <v>18</v>
       </c>
-      <c r="E9" t="s">
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="E10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" t="s">
-        <v>39</v>
-      </c>
-      <c r="E12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>21</v>
       </c>
-      <c r="C13" t="s">
+      <c r="E13" t="s">
         <v>22</v>
       </c>
-      <c r="E13" t="s">
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>24</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" t="s">
         <v>25</v>
       </c>
-      <c r="E14" t="s">
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>27</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>28</v>
       </c>
-      <c r="E15" t="s">
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>30</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" t="s">
         <v>31</v>
-      </c>
-      <c r="E16" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>